<commit_message>
added crud backend JenisIdDokumen
</commit_message>
<xml_diff>
--- a/ref/Referensi-Jabatan-Struktural-unor-id.xlsx
+++ b/ref/Referensi-Jabatan-Struktural-unor-id.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/dinaskominfo/kiken/Project/next/e-office2026/ref/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B84ABF02-DA11-4B43-B4E2-9ADFF2E3F09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8378C1D0-8250-6E44-97F9-CBCBF43DBDAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9669,7 +9669,7 @@
     <col min="1" max="2" width="36.6640625" customWidth="1"/>
     <col min="3" max="3" width="77.1640625" customWidth="1"/>
     <col min="4" max="4" width="55.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.33203125" customWidth="1"/>
     <col min="6" max="6" width="33.1640625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.1640625" bestFit="1" customWidth="1"/>
   </cols>

</xml_diff>